<commit_message>
fix(register): resolve registration buttons syntax error, unify theme mode button across all portals, add system functions doc, and add worldwide sharing launcher
</commit_message>
<xml_diff>
--- a/unused/project_gantt_chart.xlsx
+++ b/unused/project_gantt_chart.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AD19"/>
+  <dimension ref="A2:AJ22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -566,7 +566,7 @@
     <col width="44" customWidth="1" min="4" max="4"/>
     <col width="36" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="4.2" customWidth="1" min="7" max="30"/>
+    <col width="4.2" customWidth="1" min="7" max="36"/>
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1">
@@ -579,7 +579,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Gantt Chart  |  Solo Project: Sep 09 – Oct 02, 2026</t>
+          <t>Gantt Chart  |  Solo Project: Sep 09 – Oct 08, 2026</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>DAILY GANTT BARS (SEP 9 → OCT 2)</t>
+          <t>DAILY GANTT BARS (SEP 9 → OCT 8)</t>
         </is>
       </c>
       <c r="H5" s="5" t="n"/>
@@ -771,6 +771,36 @@
           <t>2</t>
         </is>
       </c>
+      <c r="AE6" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AF6" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AG6" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AH6" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AI6" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AJ6" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
@@ -1427,7 +1457,7 @@
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Oct 02 (Today)</t>
+          <t>Oct 02</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
@@ -1484,13 +1514,203 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="10" customHeight="1"/>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
-        <is>
-          <t>Solo Independent Project  |  100% Self-Implemented  |  No Outside Sources</t>
-        </is>
-      </c>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Oct 07</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>1 d</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Admin workflow and history cleanup</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Consolidated duplicate profile and intake entry points into the Registrar Desk; removed record-version controls and the release-history panel.</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>Solo implementation: keep one review workflow and simplify the command-center navigation.</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>Finished</t>
+        </is>
+      </c>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="14"/>
+      <c r="L19" s="14"/>
+      <c r="M19" s="14"/>
+      <c r="N19" s="14"/>
+      <c r="O19" s="14"/>
+      <c r="P19" s="14"/>
+      <c r="Q19" s="14"/>
+      <c r="R19" s="14"/>
+      <c r="S19" s="14"/>
+      <c r="T19" s="14"/>
+      <c r="U19" s="14"/>
+      <c r="V19" s="14"/>
+      <c r="W19" s="14"/>
+      <c r="X19" s="14"/>
+      <c r="Y19" s="14"/>
+      <c r="Z19" s="14"/>
+      <c r="AA19" s="14"/>
+      <c r="AB19" s="14"/>
+      <c r="AC19" s="14"/>
+      <c r="AD19" s="14"/>
+      <c r="AE19" s="14"/>
+      <c r="AF19" s="14"/>
+      <c r="AG19" s="14"/>
+      <c r="AH19" s="14"/>
+      <c r="AI19" s="5" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="AJ19" s="14"/>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Oct 08 (Today)</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>1 d</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Frontend separation and hosting preparation</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Moved client pages/assets into frontend/, extracted page and inline CSS, removed the dashboard operative table, updated runtime paths, and documented InfinityFree deployment constraints.</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>Solo implementation: separate backend and frontend files while preserving current routes and making hosting steps explicit.</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>Finished</t>
+        </is>
+      </c>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="14"/>
+      <c r="K20" s="14"/>
+      <c r="L20" s="14"/>
+      <c r="M20" s="14"/>
+      <c r="N20" s="14"/>
+      <c r="O20" s="14"/>
+      <c r="P20" s="14"/>
+      <c r="Q20" s="14"/>
+      <c r="R20" s="14"/>
+      <c r="S20" s="14"/>
+      <c r="T20" s="14"/>
+      <c r="U20" s="14"/>
+      <c r="V20" s="14"/>
+      <c r="W20" s="14"/>
+      <c r="X20" s="14"/>
+      <c r="Y20" s="14"/>
+      <c r="Z20" s="14"/>
+      <c r="AA20" s="14"/>
+      <c r="AB20" s="14"/>
+      <c r="AC20" s="14"/>
+      <c r="AD20" s="14"/>
+      <c r="AE20" s="14"/>
+      <c r="AF20" s="14"/>
+      <c r="AG20" s="14"/>
+      <c r="AH20" s="14"/>
+      <c r="AI20" s="14"/>
+      <c r="AJ20" s="5" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Oct 07</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>1 d</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Admin workflow and history cleanup</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Consolidated duplicate profile and intake entry points into the Registrar Desk; removed record-version controls and the release-history panel.</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>Solo implementation: keep one review workflow and simplify the command-center navigation.</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>Finished</t>
+        </is>
+      </c>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="14"/>
+      <c r="L19" s="14"/>
+      <c r="M19" s="14"/>
+      <c r="N19" s="14"/>
+      <c r="O19" s="14"/>
+      <c r="P19" s="14"/>
+      <c r="Q19" s="14"/>
+      <c r="R19" s="14"/>
+      <c r="S19" s="14"/>
+      <c r="T19" s="14"/>
+      <c r="U19" s="14"/>
+      <c r="V19" s="14"/>
+      <c r="W19" s="14"/>
+      <c r="X19" s="14"/>
+      <c r="Y19" s="14"/>
+      <c r="Z19" s="14"/>
+      <c r="AA19" s="14"/>
+      <c r="AB19" s="14"/>
+      <c r="AC19" s="14"/>
+      <c r="AD19" s="14"/>
+      <c r="AE19" s="14"/>
+      <c r="AF19" s="14"/>
+      <c r="AG19" s="14"/>
+      <c r="AH19" s="14"/>
+      <c r="AI19" s="5" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="AJ19" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1500,7 +1720,7 @@
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="F5:F6"/>
-    <mergeCell ref="G5:AD5"/>
+    <mergeCell ref="G5:AJ5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>